<commit_message>
New Sheets Alert! participatingAgencies05012025am.xlsx and pendingAgencies04302025pm.xlsx
</commit_message>
<xml_diff>
--- a/Total pendingAgencies/Total-pendingAgencies04302025pm.xlsx
+++ b/Total pendingAgencies/Total-pendingAgencies04302025pm.xlsx
@@ -436,22 +436,22 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>SUPPORT TYPE</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>COUNTY</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TYPE</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>LAW ENFORCEMENT AGENCY</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>COUNTY</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>TYPE</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>SUPPORT TYPE</t>
         </is>
       </c>
     </row>
@@ -463,7 +463,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Apopka Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -474,7 +474,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Apopka Police Department</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Atlantis Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -497,7 +497,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Atlantis Police Department</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Auburndale Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -520,7 +520,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Auburndale Police Department</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Belle Isle Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -543,7 +543,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Belle Isle Police Department</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cape Coral Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -566,7 +566,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Cape Coral Police Department</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cocoa Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -589,7 +589,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Cocoa Police Department</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Eatonville Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -612,7 +612,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Eatonville Police Department</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Edgewater Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -635,7 +635,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Edgewater Police Department</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fellsmere Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -658,7 +658,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Fellsmere Police Department</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Florida Department of Agriculture</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Florida Department of Agriculture</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Florida Department of Environmental Protection</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -704,7 +704,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Florida Department of Environmental Protection</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Florida Division of Alcoholic Beverages and Tobacco</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -727,7 +727,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Florida Division of Alcoholic Beverages and Tobacco</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Florida Gaming Control Commission</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Florida Gaming Control Commission</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Florida Gulf Coast University Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -773,7 +773,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Florida Gulf Coast University Police Department</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Florida International University Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -796,7 +796,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Florida International University Police Department</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Florida Polytechnic University Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Florida Polytechnic University Police Department</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Gulf Breeze Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -842,7 +842,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Gulf Breeze Police Department</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Hialeah Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -865,7 +865,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Hialeah Police Department</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Indialantic Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -888,7 +888,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Indialantic Police Department</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kissimmee Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -911,7 +911,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Kissimmee Police Department</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Lakeland Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -934,7 +934,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Lakeland Police Department</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Longboat Key Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -957,7 +957,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Longboat Key Police Department</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Melbourne Beach Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -980,7 +980,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Melbourne Beach Police Department</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>New Port Richey Polce Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>New Port Richey Polce Department</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>North Port Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>North Port Police Department</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ocala Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Ocala Police Department</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ocoee Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Ocoee Police Department</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Palm Springs Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Palm Springs Police Department</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Rockledge Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Rockledge Police Department</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sanford Airport Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Sanford Airport Police Department</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sanford Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Sanford Police Department</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Satellite Beach Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Satellite Beach Police Department</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>South Daytona Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>South Daytona Police Department</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>University of North Florida Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>University of North Florida Police Department</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>West Melbourne Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>West Melbourne Police Department</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>West Palm Beach Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>West Palm Beach Police Department</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Windermere Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Windermere Police Department</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Winter Springs Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Winter Springs Police Department</t>
         </is>
       </c>
     </row>
@@ -1337,22 +1337,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Forsyth County</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
           <t>Forsyth County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Forsyth County</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1364,22 +1364,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Glynn County</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
           <t>Glynn County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Glynn County</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1391,22 +1391,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Madison County</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
           <t>Madison County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Madison County</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1418,7 +1418,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Monroe Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Monroe Police Department</t>
         </is>
       </c>
     </row>
@@ -1441,22 +1441,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>Jail Enforcement Model</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Montgomery County</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
           <t>Montgomery County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Montgomery County</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Jail Enforcement Model</t>
         </is>
       </c>
     </row>
@@ -1468,22 +1468,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>Jail Enforcement Model</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Murray County</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
           <t>Murray County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Murray County</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Jail Enforcement Model</t>
         </is>
       </c>
     </row>
@@ -1495,22 +1495,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>Jail Enforcement Model</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Spalding County</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
           <t>Spalding County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Spalding County</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Jail Enforcement Model</t>
         </is>
       </c>
     </row>
@@ -1522,22 +1522,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Roscommon County</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
           <t>Roscommon County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Roscommon County</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -1549,22 +1549,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Christian County</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
           <t>Christian County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Christian County</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -1576,22 +1576,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Cascade County</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
           <t>Cascade County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Cascade County</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1603,22 +1603,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Sarpy County</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
           <t xml:space="preserve">Sarpy County Department of Corrections  </t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Sarpy County</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1630,22 +1630,22 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Carteret County</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
           <t>Cartert County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Carteret County</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1657,22 +1657,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Lincoln County</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
           <t>Lincoln County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Lincoln County</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Oklahoma Department of Corrections</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -1695,7 +1695,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Oklahoma Department of Corrections</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1707,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Oklahoma Department of Corrections</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Oklahoma Department of Corrections</t>
         </is>
       </c>
     </row>
@@ -1730,22 +1730,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Bucks County</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
           <t>Bucks County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Bucks County</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -1757,22 +1757,22 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Coke County</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
           <t>Coke County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Coke County</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -1784,22 +1784,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>Jail Enforcement Model</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Denton County</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
           <t>Denton County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Denton County</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Jail Enforcement Model</t>
         </is>
       </c>
     </row>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Hood County</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
           <t>Hood County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Hood County</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1838,22 +1838,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>San Jacinto County</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
           <t>San Jacinto County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>San Jacinto County</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Utah Department of Corrections</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Utah Department of Corrections</t>
         </is>
       </c>
     </row>
@@ -1888,22 +1888,22 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Waukesha County</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
           <t>Waukesha County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Waukesha County</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1915,22 +1915,22 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Laramie County</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
           <t>Laramie County Sheriff’s Office</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Laramie County</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -1942,22 +1942,22 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Sweetwater County</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
           <t>Sweetwater County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Sweetwater County</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Camden Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Camden Police Department</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Bartow Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Bartow Police Department</t>
         </is>
       </c>
     </row>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Daytona Beach Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Daytona Beach Police Department</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Lake City Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Lake City Police Department</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Lake Clark Shores Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Lake Clark Shores Police Department</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Melbourne International Airport Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Melbourne International Airport Police Department</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Riviera Beach Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Riviera Beach Police Department</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Heritage Creek Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Heritage Creek Police Department</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Taylor Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Taylor Police Department</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Saint Mary Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Saint Mary Police Department</t>
         </is>
       </c>
     </row>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Damascus County</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
           <t>Damascus County Constable</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Damascus County</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -2226,22 +2226,22 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Sumner County</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
           <t>Sumner County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Sumner County</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -2253,22 +2253,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crenshaw County </t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
           <t>Crenshaw County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Crenshaw County </t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -2280,22 +2280,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Navajo County</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
           <t>Navajo County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Navajo County</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Alachua Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Alachua Police Department</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Blountstown Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Blountstown Police Department</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>City of Hialeah Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
@@ -2364,7 +2364,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>City of Hialeah Police Department</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Edgewood Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Edgewood Police Department</t>
         </is>
       </c>
     </row>
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Green Cove Springs Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Green Cove Springs Police Department</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Havana Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C83" t="inlineStr"/>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Havana Police Department</t>
         </is>
       </c>
     </row>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Highland Beach Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Highland Beach Police Department</t>
         </is>
       </c>
     </row>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Holmes Beach Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C85" t="inlineStr"/>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Holmes Beach Police Department</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Indian Harbour Beach Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Indian Harbour Beach Police Department</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Key Colony Beach Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Key Colony Beach Police Department</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Lady Lake Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C88" t="inlineStr"/>
@@ -2548,7 +2548,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Lady Lake Police Department</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Lantana Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C89" t="inlineStr"/>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Lantana Police Department</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Live Oak Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
@@ -2594,7 +2594,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Live Oak Police Department</t>
         </is>
       </c>
     </row>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Longwood Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Longwood Police Department</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Melbourne Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C92" t="inlineStr"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Melbourne Police Department</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Ocean Ridge Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Ocean Ridge Police Department</t>
         </is>
       </c>
     </row>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Orange City Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Orange City Police Department</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Ormond Beach Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Ormond Beach Police Department</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Pembroke Park Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Pembroke Park Police Department</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2744,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Pembroke Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Pembroke Police Department</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ponce Inlet Police Department </t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C98" t="inlineStr"/>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t xml:space="preserve">Ponce Inlet Police Department </t>
         </is>
       </c>
     </row>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Sebastian Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Sebastian Police Department</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Sewalls Point Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C100" t="inlineStr"/>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Sewalls Point Police Department</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>St. Cloud Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C101" t="inlineStr"/>
@@ -2847,7 +2847,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>St. Cloud Police Department</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Stuart Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C102" t="inlineStr"/>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Stuart Police Department</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Zephyrhills Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C103" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Zephyrhills Police Department</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>City of Monroe Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C104" t="inlineStr"/>
@@ -2916,7 +2916,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>City of Monroe Police Department</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Greens Fork Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C105" t="inlineStr"/>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Greens Fork Police Department</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Monmouth Winthrop Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C106" t="inlineStr"/>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Monmouth Winthrop Police Department</t>
         </is>
       </c>
     </row>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Candia Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C107" t="inlineStr"/>
@@ -2985,7 +2985,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Candia Police Department</t>
         </is>
       </c>
     </row>
@@ -2997,7 +2997,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>New Hampshire State Police</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C108" t="inlineStr"/>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>New Hampshire State Police</t>
         </is>
       </c>
     </row>
@@ -3020,22 +3020,22 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Muskogee County</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
           <t>Muskogee County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Muskogee County</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -3047,22 +3047,22 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Kershaw County</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
           <t>Kershaw County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>Kershaw County</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -3074,22 +3074,22 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Giles County</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
           <t>Giles County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>Giles County</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -3101,22 +3101,22 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Austin County</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
           <t>Austin County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Austin County</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -3128,22 +3128,22 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Burleson County</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
           <t>Burleson County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>Burleson County</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -3155,22 +3155,22 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
+          <t>Jail Enforcement Model</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Ellis County</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
           <t>Ellis County Sheriff’s Office</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>Ellis County</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Jail Enforcement Model</t>
         </is>
       </c>
     </row>
@@ -3182,22 +3182,22 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Hamilton County</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
           <t xml:space="preserve">Hamilton County Sheriff's Office </t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Hamilton County</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -3209,22 +3209,22 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Live Oak County</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
           <t>Live Oak County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Live Oak County</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -3236,22 +3236,22 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Terrell County</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
           <t>Terrell County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>Terrell County</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -3263,22 +3263,22 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Wichita County</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
           <t>Wichita County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>Wichita County</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -3290,22 +3290,22 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Winkler County</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
           <t>Winkler County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>Winkler County</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -3317,22 +3317,22 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shenandoah County </t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
           <t>Shenandoah County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Shenandoah County </t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -3344,22 +3344,22 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Smyth County</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
           <t>Smyth County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Smyth County</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Alachua County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Alachua County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Gilchrist County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
@@ -3405,7 +3405,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Gilchrist County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Glades County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -3428,7 +3428,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Glades County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Hardee County Sheriff’s Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Hardee County Sheriff’s Office</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Hillsborough County Sheriff’s Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C126" t="inlineStr"/>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Hillsborough County Sheriff’s Office</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Jackson County Correctional Facility</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Jackson County Correctional Facility</t>
         </is>
       </c>
     </row>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Lee County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C128" t="inlineStr"/>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Lee County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miami-Dade County Corrections and Rehabilitation </t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C129" t="inlineStr"/>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t xml:space="preserve">Miami-Dade County Corrections and Rehabilitation </t>
         </is>
       </c>
     </row>
@@ -3555,7 +3555,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Orange County Sheriff’s Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
@@ -3566,7 +3566,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Orange County Sheriff’s Office</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Palm Beach County Sheriff’s Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
@@ -3589,7 +3589,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Palm Beach County Sheriff’s Office</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Pasco County Jail</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Pasco County Jail</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Union County Sheriff’s Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C133" t="inlineStr"/>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Union County Sheriff’s Office</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Washington County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C134" t="inlineStr"/>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Washington County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3670,7 +3670,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Columbia County Sheriff’s Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Columbia County Sheriff’s Office</t>
         </is>
       </c>
     </row>
@@ -3693,7 +3693,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Monroe County Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C136" t="inlineStr"/>
@@ -3704,7 +3704,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Monroe County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3716,7 +3716,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Spaulding County Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Spaulding County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3739,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Walker County Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
@@ -3750,7 +3750,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Walker County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3762,7 +3762,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Bossier Parish Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
@@ -3773,7 +3773,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Bossier Parish Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3785,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Carroll County Sheriff’s Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Carroll County Sheriff’s Office</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Nassau County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Nassau County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Butler County Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
@@ -3842,7 +3842,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Butler County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Logan County Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C143" t="inlineStr"/>
@@ -3865,7 +3865,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Logan County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3877,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Okmulgee County Criminal Justice Authority</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
@@ -3888,7 +3888,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Okmulgee County Criminal Justice Authority</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Franklin County Sheriff’s Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C145" t="inlineStr"/>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Franklin County Sheriff’s Office</t>
         </is>
       </c>
     </row>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Hamilton County Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Hamilton County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3946,7 +3946,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Putnam County Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C147" t="inlineStr"/>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Putnam County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3969,7 +3969,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Bee County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C148" t="inlineStr"/>
@@ -3980,7 +3980,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Bee County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -3992,7 +3992,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Grayson County Sheriff’s Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C149" t="inlineStr"/>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Grayson County Sheriff’s Office</t>
         </is>
       </c>
     </row>
@@ -4015,7 +4015,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Gregg County Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C150" t="inlineStr"/>
@@ -4026,7 +4026,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Gregg County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>San Jacinto County Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C151" t="inlineStr"/>
@@ -4049,7 +4049,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>San Jacinto County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Victoria County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C152" t="inlineStr"/>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Victoria County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Campbell County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C153" t="inlineStr"/>
@@ -4095,7 +4095,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Campbell County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4107,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Sweetwater County Sheriff’s Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Sweetwater County Sheriff’s Office</t>
         </is>
       </c>
     </row>
@@ -4130,7 +4130,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Elmore County Sheriff's Office</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C155" t="inlineStr"/>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Elmore County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4153,7 +4153,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Florida State Guard</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
@@ -4164,7 +4164,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Florida State Guard</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Jasper County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
@@ -4187,7 +4187,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Jasper County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Mineral County Sheriff's Office</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Mineral County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4222,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Portage County Sheriff's Office</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Portage County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4245,7 +4245,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Portage County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Portage County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4268,7 +4268,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Minehaha County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Minehaha County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4291,7 +4291,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Deaf Smith County Sheriff's Office</t>
+          <t>Warrant Service Officer</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Warrant Service Officer</t>
+          <t>Deaf Smith County Sheriff's Office</t>
         </is>
       </c>
     </row>
@@ -4314,22 +4314,22 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
+          <t>Jail Enforcement Model</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Henry County</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
           <t>Henry County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>Henry County</t>
-        </is>
-      </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E163" t="inlineStr">
-        <is>
-          <t>Jail Enforcement Model</t>
         </is>
       </c>
     </row>
@@ -4341,22 +4341,22 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Henry County</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
           <t>Henry County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>Henry County</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Okeechobee Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -4379,7 +4379,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Okeechobee Police Department</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Tavares Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Tavares Police Department</t>
         </is>
       </c>
     </row>
@@ -4414,7 +4414,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Venice Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -4425,7 +4425,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Venice Police Department</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4437,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Kenner Police Department</t>
+          <t>Jail Enforcement Model</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Jail Enforcement Model</t>
+          <t>Kenner Police Department</t>
         </is>
       </c>
     </row>
@@ -4460,7 +4460,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Mississippi Attorney General's Office</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Mississippi Attorney General's Office</t>
         </is>
       </c>
     </row>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Troy Police Department</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Troy Police Department</t>
         </is>
       </c>
     </row>
@@ -4506,22 +4506,22 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Minnehaha County</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
           <t>Minnehaha County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>Minnehaha County</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E171" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -4533,22 +4533,22 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>McKenzie County</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
           <t>McKenzie County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>McKenzie County</t>
-        </is>
-      </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E172" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -4560,22 +4560,22 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Wood County</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
           <t>Wood County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>Wood County</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -4587,22 +4587,22 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Lancaster County</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
           <t>Lancaster County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>Lancaster County</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -4614,22 +4614,22 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Panola County</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
           <t>Panola County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>Panola County</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -4641,22 +4641,22 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
+          <t>Warrant Service Officer</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Loudoun County</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
           <t>Loudoun County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>Loudoun County</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>Warrant Service Officer</t>
         </is>
       </c>
     </row>
@@ -4668,22 +4668,22 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>York County</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Municipality</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
           <t>Wells Police Department</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>York County</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>Municipality</t>
-        </is>
-      </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -4695,22 +4695,22 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
+          <t>Task Force Model</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Kershaw County</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
           <t>Kershaw County Sheriff's Office</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>Kershaw County</t>
-        </is>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>County</t>
-        </is>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>Task Force Model</t>
         </is>
       </c>
     </row>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Texas National Guard</t>
+          <t>Task Force Model</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Task Force Model</t>
+          <t>Texas National Guard</t>
         </is>
       </c>
     </row>

</xml_diff>